<commit_message>
larger patch size 32
</commit_message>
<xml_diff>
--- a/manual_grid_search.xlsx
+++ b/manual_grid_search.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brenden/Desktop/motorVAE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66A33F30-8883-464B-A663-0A5EA03C1F1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7443669F-B64D-E042-86D2-FACA8FBC901D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14760" yWindow="900" windowWidth="14480" windowHeight="17080" xr2:uid="{81F0242E-9469-2D43-9768-647BA0AB9CA2}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
   <si>
     <t>Notes</t>
   </si>
@@ -129,6 +129,12 @@
   </si>
   <si>
     <t>Smaller batch size=53;</t>
+  </si>
+  <si>
+    <t>res256_lat128_ep100_bat71_lrn0.0002_rec100.0_per5.0_gan0.2_kld0.1(tc0.002_mi0.1_dk2e-05)_cls0.2_pat16</t>
+  </si>
+  <si>
+    <t>Higher learning rate=0.0002;</t>
   </si>
 </sst>
 </file>
@@ -198,7 +204,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -255,13 +261,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -337,6 +366,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -674,194 +710,200 @@
   <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="51.6640625" style="7" customWidth="1"/>
-    <col min="3" max="3" width="46.33203125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="35" style="4" customWidth="1"/>
-    <col min="5" max="5" width="27.6640625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="34" style="4" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="10.83203125" style="4"/>
+    <col min="1" max="1" width="11.6640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.6640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="35" style="3" customWidth="1"/>
+    <col min="5" max="5" width="27.6640625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="34" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="10.83203125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="A2" s="9">
+      <c r="A2" s="8">
         <v>61150792</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="3"/>
-    </row>
-    <row r="3" spans="1:5" s="13" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A3" s="11">
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:5" s="12" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A3" s="10">
         <v>61454092</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="13" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="18" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A4" s="16">
+    <row r="4" spans="1:5" s="17" customFormat="1" ht="42" x14ac:dyDescent="0.2">
+      <c r="A4" s="15">
         <v>61454513</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="19"/>
-    </row>
-    <row r="5" spans="1:5" s="22" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A5" s="20">
+      <c r="E4" s="18"/>
+    </row>
+    <row r="5" spans="1:5" s="21" customFormat="1" ht="42" x14ac:dyDescent="0.2">
+      <c r="A5" s="19">
         <v>61454535</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="21" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="22" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A6" s="23">
+    <row r="6" spans="1:5" s="21" customFormat="1" ht="42" x14ac:dyDescent="0.2">
+      <c r="A6" s="22">
         <v>61454554</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="21" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="26" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A7" s="24">
+    <row r="7" spans="1:5" s="25" customFormat="1" ht="42" x14ac:dyDescent="0.2">
+      <c r="A7" s="23">
         <v>61454567</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="C7" s="25" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="28" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A8" s="27">
+    <row r="8" spans="1:5" s="27" customFormat="1" ht="42" x14ac:dyDescent="0.2">
+      <c r="A8" s="26">
         <v>61454652</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="27" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:5" s="30" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A9" s="29">
+    <row r="9" spans="1:5" s="29" customFormat="1" ht="42" x14ac:dyDescent="0.2">
+      <c r="A9" s="28">
         <v>61454690</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="29" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="28" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A10" s="27">
+    <row r="10" spans="1:5" s="27" customFormat="1" ht="42" x14ac:dyDescent="0.2">
+      <c r="A10" s="26">
         <v>61454935</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="C10" s="27" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:5" s="31" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A11" s="32">
+    <row r="11" spans="1:5" s="30" customFormat="1" ht="42" x14ac:dyDescent="0.2">
+      <c r="A11" s="31">
         <v>61454936</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="31" t="s">
+      <c r="C11" s="30" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="30" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A12" s="29">
+    <row r="12" spans="1:5" s="29" customFormat="1" ht="42" x14ac:dyDescent="0.2">
+      <c r="A12" s="28">
         <v>61454938</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="30" t="s">
+      <c r="C12" s="29" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
+    <row r="13" spans="1:5" s="34" customFormat="1" ht="42" x14ac:dyDescent="0.2">
+      <c r="A13" s="32">
         <v>61455038</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="34" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="B14" s="15" t="s">
+    <row r="14" spans="1:5" s="34" customFormat="1" ht="42" x14ac:dyDescent="0.2">
+      <c r="A14" s="32">
+        <v>61455094</v>
+      </c>
+      <c r="B14" s="33" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="34" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+      <c r="B15" s="14" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="B15" s="15" t="s">
-        <v>6</v>
-      </c>
-    </row>
     <row r="16" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="B16" s="15" t="s">
+      <c r="B16" s="14" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
smaller latent space 96
</commit_message>
<xml_diff>
--- a/manual_grid_search.xlsx
+++ b/manual_grid_search.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brenden/Desktop/motorVAE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7443669F-B64D-E042-86D2-FACA8FBC901D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02871369-3C25-DF42-A003-98E207D8B750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14760" yWindow="900" windowWidth="14480" windowHeight="17080" xr2:uid="{81F0242E-9469-2D43-9768-647BA0AB9CA2}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="35">
   <si>
     <t>Notes</t>
   </si>
@@ -135,6 +135,12 @@
   </si>
   <si>
     <t>Higher learning rate=0.0002;</t>
+  </si>
+  <si>
+    <t>Larger patch size=32;</t>
+  </si>
+  <si>
+    <t>res256_lat128_ep100_bat71_lrn0.0001_rec100.0_per5.0_gan0.2_kld0.1(tc0.002_mi0.1_dk2e-05)_cls0.2_pat32</t>
   </si>
 </sst>
 </file>
@@ -204,7 +210,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -261,35 +267,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -366,13 +348,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -707,7 +682,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{061CEEAB-0DCA-3847-86A8-898871078FB7}">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.6640625" style="9" bestFit="1" customWidth="1"/>
@@ -864,46 +839,57 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="29" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A12" s="28">
+    <row r="12" spans="1:5" s="30" customFormat="1" ht="42" x14ac:dyDescent="0.2">
+      <c r="A12" s="31">
         <v>61454938</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="C12" s="30" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:5" s="34" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A13" s="32">
+    <row r="13" spans="1:5" s="27" customFormat="1" ht="42" x14ac:dyDescent="0.2">
+      <c r="A13" s="26">
         <v>61455038</v>
       </c>
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="34" t="s">
+      <c r="C13" s="27" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:5" s="34" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A14" s="32">
+    <row r="14" spans="1:5" s="30" customFormat="1" ht="42" x14ac:dyDescent="0.2">
+      <c r="A14" s="31">
         <v>61455094</v>
       </c>
-      <c r="B14" s="33" t="s">
+      <c r="B14" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="34" t="s">
+      <c r="C14" s="30" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="B15" s="14" t="s">
-        <v>6</v>
+    <row r="15" spans="1:5" s="29" customFormat="1" ht="42" x14ac:dyDescent="0.2">
+      <c r="A15" s="28">
+        <v>61455158</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="29" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="B16" s="14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" ht="42" x14ac:dyDescent="0.2">
+      <c r="B17" s="14" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed kld and new benchmark parameters
</commit_message>
<xml_diff>
--- a/manual_grid_search.xlsx
+++ b/manual_grid_search.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brenden/Desktop/motorVAE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BA92D90-D579-A143-A438-CF55BC5C7260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF6443DC-22CF-5B47-B89A-C1EE8E68490B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="900" windowWidth="14440" windowHeight="17080" xr2:uid="{81F0242E-9469-2D43-9768-647BA0AB9CA2}"/>
+    <workbookView xWindow="160" yWindow="900" windowWidth="15500" windowHeight="17060" xr2:uid="{81F0242E-9469-2D43-9768-647BA0AB9CA2}"/>
   </bookViews>
   <sheets>
     <sheet name="May 20" sheetId="1" r:id="rId1"/>
+    <sheet name="May 21" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="46">
   <si>
     <t>Notes</t>
   </si>
@@ -150,6 +151,30 @@
   </si>
   <si>
     <t>Lower kld loss 0.1; stable GAN at 0.2;</t>
+  </si>
+  <si>
+    <t>Reconstructions are sharp; Samples don't look like real cars; total correlation loss is negative;</t>
+  </si>
+  <si>
+    <t>kld might be too low, resulting in poor samples; fix total correlation loss;</t>
+  </si>
+  <si>
+    <t>Reconstructions looks poor and similar to each other;</t>
+  </si>
+  <si>
+    <t>GAN weight too high, causing reconstructions to look similar in order to trick discriminator;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Good reconstructions, comparable to when kld=0.1; The samples look a bit more like real cars than when kld=0.1; </t>
+  </si>
+  <si>
+    <t>Still need to fix the random samples; Fix negative TC loss;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Good reconstructions; Samples look more like real cars; </t>
+  </si>
+  <si>
+    <t>Fix negative TC loss;</t>
   </si>
 </sst>
 </file>
@@ -341,9 +366,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -761,8 +786,8 @@
       </c>
       <c r="E4" s="15"/>
     </row>
-    <row r="5" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="A5" s="8">
+    <row r="5" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A5" s="24">
         <v>61532163</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -771,10 +796,16 @@
       <c r="C5" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="A6" s="23">
-        <v>61497566</v>
+      <c r="D5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A6" s="24">
+        <v>61551107</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>15</v>
@@ -782,10 +813,16 @@
       <c r="C6" s="3" t="s">
         <v>14</v>
       </c>
+      <c r="D6" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="7" spans="1:5" s="18" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A7" s="23">
-        <v>61497680</v>
+      <c r="A7" s="22">
+        <v>61551110</v>
       </c>
       <c r="B7" s="17" t="s">
         <v>13</v>
@@ -795,8 +832,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" s="14" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A8" s="23">
-        <v>61497723</v>
+      <c r="A8" s="22">
+        <v>61551118</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>18</v>
@@ -817,8 +854,8 @@
       </c>
     </row>
     <row r="10" spans="1:5" s="14" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A10" s="23">
-        <v>61497826</v>
+      <c r="A10" s="22">
+        <v>61551123</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>21</v>
@@ -828,7 +865,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="A11" s="24">
+      <c r="A11" s="23">
         <v>61457023</v>
       </c>
       <c r="B11" s="5" t="s">
@@ -838,9 +875,9 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="18" customFormat="1" ht="42" x14ac:dyDescent="0.2">
-      <c r="A12" s="23">
-        <v>61497846</v>
+    <row r="12" spans="1:5" s="18" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A12" s="24">
+        <v>61551134</v>
       </c>
       <c r="B12" s="17" t="s">
         <v>24</v>
@@ -848,10 +885,16 @@
       <c r="C12" s="18" t="s">
         <v>25</v>
       </c>
+      <c r="D12" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="13" spans="1:5" s="14" customFormat="1" ht="42" x14ac:dyDescent="0.2">
       <c r="A13" s="22">
-        <v>61457105</v>
+        <v>61551147</v>
       </c>
       <c r="B13" s="13" t="s">
         <v>27</v>
@@ -861,14 +904,20 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="A14" s="23">
-        <v>61497930</v>
+      <c r="A14" s="24">
+        <v>61551174</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>29</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>30</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -902,6 +951,67 @@
       <c r="B18" s="5" t="s">
         <v>6</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DB3904B-14D6-7B45-AF76-FEBD469BA2AA}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.6640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.6640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="35" style="3" customWidth="1"/>
+    <col min="5" max="5" width="27.6640625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="34" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="10.83203125" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+      <c r="A2" s="8">
+        <v>61150792</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
highest learning rate 0.0003
</commit_message>
<xml_diff>
--- a/manual_grid_search.xlsx
+++ b/manual_grid_search.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brenden/Desktop/motorVAE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197DAEE4-CA0D-7D4D-9C93-BCF8FF05A1D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57027276-677A-554A-A0B3-0051EDD39D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="160" yWindow="900" windowWidth="15500" windowHeight="17060" activeTab="1" xr2:uid="{81F0242E-9469-2D43-9768-647BA0AB9CA2}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="54">
   <si>
     <t>Notes</t>
   </si>
@@ -184,6 +184,21 @@
   </si>
   <si>
     <t>Lower kld 0.3;</t>
+  </si>
+  <si>
+    <t>res256_lat128_ep100_bat71_lrn0.00018_rec100.0_per5.0_gan0.5_kld0.3(tc0.002_mi0.1_dk2e-05)_cls0.2_pat16</t>
+  </si>
+  <si>
+    <t>res256_lat128_ep100_bat71_lrn0.00018_rec100.0_per5.0_gan0.5_kld0.7(tc0.002_mi0.1_dk2e-05)_cls0.2_pat16</t>
+  </si>
+  <si>
+    <t>Higher kld 0.7;</t>
+  </si>
+  <si>
+    <t>Higher learning rate = 0.0002</t>
+  </si>
+  <si>
+    <t>Highest learning rate = 0.0003</t>
   </si>
 </sst>
 </file>
@@ -1026,9 +1041,11 @@
       <c r="E2" s="12"/>
     </row>
     <row r="3" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="A3" s="8"/>
+      <c r="A3" s="8">
+        <v>61619125</v>
+      </c>
       <c r="B3" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>48</v>
@@ -1036,9 +1053,14 @@
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="A4" s="8"/>
+      <c r="A4" s="8">
+        <v>61619127</v>
+      </c>
       <c r="B4" s="5" t="s">
-        <v>47</v>
+        <v>50</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -1046,11 +1068,17 @@
       <c r="B5" s="5" t="s">
         <v>47</v>
       </c>
+      <c r="C5" s="3" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="6" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A6" s="8"/>
       <c r="B6" s="5" t="s">
         <v>47</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="42" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
best fit param, more epochs
</commit_message>
<xml_diff>
--- a/manual_grid_search.xlsx
+++ b/manual_grid_search.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brenden/Desktop/motorVAE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57027276-677A-554A-A0B3-0051EDD39D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C100AD-EEC8-BA49-A7CE-99BF1CC9FA6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="160" yWindow="900" windowWidth="15500" windowHeight="17060" activeTab="1" xr2:uid="{81F0242E-9469-2D43-9768-647BA0AB9CA2}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="56">
   <si>
     <t>Notes</t>
   </si>
@@ -199,6 +199,12 @@
   </si>
   <si>
     <t>Highest learning rate = 0.0003</t>
+  </si>
+  <si>
+    <t>res256_lat128_ep100_bat71_lrn0.0002_rec100.0_per5.0_gan0.5_kld0.5(tc0.002_mi0.1_dk2e-05)_cls0.2_pat16</t>
+  </si>
+  <si>
+    <t>res256_lat128_ep100_bat71_lrn0.0003_rec100.0_per5.0_gan0.5_kld0.5(tc0.002_mi0.1_dk2e-05)_cls0.2_pat16</t>
   </si>
 </sst>
 </file>
@@ -1064,18 +1070,22 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="A5" s="8"/>
+      <c r="A5" s="8">
+        <v>61619203</v>
+      </c>
       <c r="B5" s="5" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="A6" s="8"/>
+      <c r="A6" s="8">
+        <v>61619210</v>
+      </c>
       <c r="B6" s="5" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>53</v>

</xml_diff>

<commit_message>
batch 100, epoch 180
</commit_message>
<xml_diff>
--- a/manual_grid_search.xlsx
+++ b/manual_grid_search.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brenden/Desktop/motorVAE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE82FC90-AE0D-3B4F-A834-7AFC72A0FE35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F215FA8C-302D-2445-B7F6-4E14B7A53D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15060" yWindow="920" windowWidth="14200" windowHeight="17060" activeTab="4" xr2:uid="{81F0242E-9469-2D43-9768-647BA0AB9CA2}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="82">
   <si>
     <t>Notes</t>
   </si>
@@ -283,6 +283,9 @@
   </si>
   <si>
     <t>res256_lat128_ep100_bat142_lrn0.0001_rec125.0_per5.0_gan0.2_kld0.1(tc0.1_mi0.1_dk2e-05)_cls0.2_pat16</t>
+  </si>
+  <si>
+    <t>Total loss started increasing after 40 epochs, probably due to KL loss… but KL loss isnt decreasing.</t>
   </si>
 </sst>
 </file>
@@ -1476,7 +1479,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="68" x14ac:dyDescent="0.2">
       <c r="A2" s="26">
         <v>16697</v>
       </c>
@@ -1488,6 +1491,9 @@
       </c>
       <c r="D2" s="3" t="s">
         <v>76</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -1503,7 +1509,7 @@
     </row>
     <row r="4" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A4" s="8">
-        <v>18317</v>
+        <v>18493</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>80</v>

</xml_diff>

<commit_message>
working checkpoint before adding sales network
</commit_message>
<xml_diff>
--- a/manual_grid_search.xlsx
+++ b/manual_grid_search.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brenden/Desktop/motorVAE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F215FA8C-302D-2445-B7F6-4E14B7A53D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42CD6BA8-52D5-1C46-A2F4-61C8944BF636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15060" yWindow="920" windowWidth="14200" windowHeight="17060" activeTab="4" xr2:uid="{81F0242E-9469-2D43-9768-647BA0AB9CA2}"/>
+    <workbookView xWindow="15060" yWindow="920" windowWidth="14200" windowHeight="17060" activeTab="5" xr2:uid="{81F0242E-9469-2D43-9768-647BA0AB9CA2}"/>
   </bookViews>
   <sheets>
     <sheet name="May 20" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="May 26" sheetId="4" r:id="rId3"/>
     <sheet name="May 27" sheetId="6" r:id="rId4"/>
     <sheet name="Jun 25" sheetId="8" r:id="rId5"/>
+    <sheet name="Jul 4" sheetId="9" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="87">
   <si>
     <t>Notes</t>
   </si>
@@ -270,9 +271,6 @@
     <t>More epochs, lower kld, larger tc; migrated to H100 GPUs</t>
   </si>
   <si>
-    <t>Reconstructions are ok, but quickly devolve into one standard car. Ask Remi why.</t>
-  </si>
-  <si>
     <t>res256_lat128_ep100_bat100_lrn0.0001_rec125.0_per5.0_gan0.2_kld0.1(tc0.1_mi0.1_dk2e-05)_cls0.2_pat16</t>
   </si>
   <si>
@@ -286,6 +284,24 @@
   </si>
   <si>
     <t>Total loss started increasing after 40 epochs, probably due to KL loss… but KL loss isnt decreasing.</t>
+  </si>
+  <si>
+    <t>Reconstructions look pretty good. Samples look a little wonky, but clean up a bit towards epoch 90. More artifacts in samples than other batch sizes.</t>
+  </si>
+  <si>
+    <t>Reconstructions look great, but the samples look worse.</t>
+  </si>
+  <si>
+    <t>Reconstructions are ok.</t>
+  </si>
+  <si>
+    <t>Batch size 100 had fantastic reconstructions, with mediocre samples. Seems that with larger batch sizes, might need more epochs. I think optimal parameters are BATCH 100, EPOCHS 150+</t>
+  </si>
+  <si>
+    <t>res256_lat128_ep180_bat100_lrn0.0001_rec125.0_per5.0_gan0.2_kld0.1(tc0.1_mi0.1_dk2e-05)_cls0.2_pat16</t>
+  </si>
+  <si>
+    <t>180 epochs; 100 batch size</t>
   </si>
 </sst>
 </file>
@@ -434,7 +450,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -499,6 +515,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1440,7 +1459,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1760FD8E-E982-BC44-90D2-1A14944264FD}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.6640625" style="9" bestFit="1" customWidth="1"/>
@@ -1490,10 +1509,10 @@
         <v>75</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -1501,24 +1520,145 @@
         <v>18103</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+      <c r="D3" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="68" x14ac:dyDescent="0.2">
       <c r="A4" s="8">
         <v>18493</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>79</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B5" s="5"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" s="27"/>
+      <c r="B26" s="27"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="27"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" s="27"/>
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A25:D27"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB4B8F2A-5D9C-A041-BCB7-D7BAAD38B979}">
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.6640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.6640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="35" style="3" customWidth="1"/>
+    <col min="5" max="5" width="27.6640625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="34" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="10.83203125" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+      <c r="A2" s="8">
+        <v>69512</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="26"/>
+      <c r="B3" s="5"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="8"/>
+      <c r="B4" s="5"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B5" s="5"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" s="27"/>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" s="27"/>
+      <c r="B26" s="27"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="27"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" s="27"/>
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A25:D27"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fixed max kld w
</commit_message>
<xml_diff>
--- a/manual_grid_search.xlsx
+++ b/manual_grid_search.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brenden/Desktop/motorVAE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{261260BF-CEBA-804C-967B-C42D78D72C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C34AFA9F-E0C6-5143-B863-52179D87B437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15060" yWindow="920" windowWidth="14200" windowHeight="17060" activeTab="5" xr2:uid="{81F0242E-9469-2D43-9768-647BA0AB9CA2}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="94">
   <si>
     <t>Notes</t>
   </si>
@@ -311,6 +311,18 @@
   </si>
   <si>
     <t>Epoch down to 100; dropped final kld to 0.09; increased classification loss weight to 0.3; added sales classifier</t>
+  </si>
+  <si>
+    <t>res256_lat128_ep100_bat100_lrn0.0001_rec125.0_per5.0_gan0.2_kld1.0(tc0.1_mi0.05_dk0.0001)_cls0.3_pat16</t>
+  </si>
+  <si>
+    <t>Allow gradients to flow through KL loss components! Increased KL loss weights.</t>
+  </si>
+  <si>
+    <t>lat128_eo100_bat100_lrn0.0001_rec125_per5_gan0.2_kld0.09warm5(tc0.1_mi0.05_dk0.0001)_cls0.3</t>
+  </si>
+  <si>
+    <t>Reduced kld warmup to 5 to prevent model from committing too much to entangled representations early (should target the point where reconstruction loss flattens out).</t>
   </si>
 </sst>
 </file>
@@ -1649,12 +1661,27 @@
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="8"/>
-      <c r="B4" s="5"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B5" s="5"/>
+    <row r="4" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+      <c r="A4" s="8">
+        <v>82228</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="68" x14ac:dyDescent="0.2">
+      <c r="A5" s="8">
+        <v>82236</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="27"/>

</xml_diff>

<commit_message>
mi and dk 4
</commit_message>
<xml_diff>
--- a/manual_grid_search.xlsx
+++ b/manual_grid_search.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brenden/Desktop/motorVAE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F31D2A0D-D3E5-024C-83A4-381F5CC052AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A97B62F6-F6AE-394B-A60E-EC636BE4BD8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15060" yWindow="920" windowWidth="14200" windowHeight="17060" activeTab="5" xr2:uid="{81F0242E-9469-2D43-9768-647BA0AB9CA2}"/>
+    <workbookView xWindow="15060" yWindow="900" windowWidth="14200" windowHeight="17060" activeTab="6" xr2:uid="{81F0242E-9469-2D43-9768-647BA0AB9CA2}"/>
   </bookViews>
   <sheets>
     <sheet name="May 20" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="May 27" sheetId="6" r:id="rId4"/>
     <sheet name="Jun 25" sheetId="8" r:id="rId5"/>
     <sheet name="Jul 4" sheetId="9" r:id="rId6"/>
+    <sheet name="Jul 22" sheetId="11" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="123">
   <si>
     <t>Notes</t>
   </si>
@@ -404,6 +405,12 @@
   </si>
   <si>
     <t>Reduced epochs to 100.</t>
+  </si>
+  <si>
+    <t>Best parameters from last iteration. Running with updated sales data.</t>
+  </si>
+  <si>
+    <t>Slightly lower mi and dk to improve stability</t>
   </si>
 </sst>
 </file>
@@ -478,7 +485,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -506,6 +513,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -571,7 +584,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -637,23 +650,30 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1684,24 +1704,24 @@
       <c r="B5" s="5"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="27" t="s">
+      <c r="A25" s="32" t="s">
         <v>84</v>
       </c>
-      <c r="B25" s="27"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="27"/>
+      <c r="B25" s="32"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="27"/>
-      <c r="B26" s="27"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
+      <c r="A26" s="32"/>
+      <c r="B26" s="32"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="27"/>
-      <c r="B27" s="27"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
+      <c r="A27" s="32"/>
+      <c r="B27" s="32"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1842,14 +1862,14 @@
         <v>102</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="32" customFormat="1" ht="85" x14ac:dyDescent="0.2">
-      <c r="A8" s="30">
+    <row r="8" spans="1:5" s="31" customFormat="1" ht="85" x14ac:dyDescent="0.2">
+      <c r="A8" s="29">
         <v>83757</v>
       </c>
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="D8" s="31" t="s">
         <v>110</v>
       </c>
     </row>
@@ -1857,7 +1877,7 @@
       <c r="A9" s="8">
         <v>83786</v>
       </c>
-      <c r="B9" s="29" t="s">
+      <c r="B9" s="28" t="s">
         <v>107</v>
       </c>
       <c r="D9" s="3" t="s">
@@ -1868,7 +1888,7 @@
       <c r="A10" s="8">
         <v>83801</v>
       </c>
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="27" t="s">
         <v>108</v>
       </c>
       <c r="D10" s="3" t="s">
@@ -1879,7 +1899,7 @@
       <c r="A11" s="8">
         <v>83824</v>
       </c>
-      <c r="B11" s="28" t="s">
+      <c r="B11" s="27" t="s">
         <v>109</v>
       </c>
       <c r="C11" s="3" t="s">
@@ -1896,7 +1916,7 @@
       <c r="A12" s="8">
         <v>96291</v>
       </c>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="27" t="s">
         <v>115</v>
       </c>
       <c r="C12" s="3" t="s">
@@ -1913,7 +1933,7 @@
       <c r="A13" s="8">
         <v>109353</v>
       </c>
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="27" t="s">
         <v>119</v>
       </c>
       <c r="C13" s="3" t="s">
@@ -1921,22 +1941,22 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="27"/>
-      <c r="B25" s="27"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="27"/>
+      <c r="A25" s="32"/>
+      <c r="B25" s="32"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="27"/>
-      <c r="B26" s="27"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
+      <c r="A26" s="32"/>
+      <c r="B26" s="32"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="27"/>
-      <c r="B27" s="27"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
+      <c r="A27" s="32"/>
+      <c r="B27" s="32"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1944,4 +1964,93 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED27C2F8-E261-D740-8906-31762EE757F4}">
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.6640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.6640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="46.33203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="35" style="3" customWidth="1"/>
+    <col min="5" max="5" width="27.6640625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="34" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="10.83203125" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" s="36" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A2" s="34">
+        <v>353433</v>
+      </c>
+      <c r="B2" s="35" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" s="36" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.2">
+      <c r="A3" s="8">
+        <v>353427</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="32"/>
+      <c r="B14" s="32"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="32"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="32"/>
+      <c r="B15" s="32"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="32"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="32"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A14:D16"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>